<commit_message>
chore(watchlist): 미국 주도주 리스트 2026-08-26
</commit_message>
<xml_diff>
--- a/watchlist_us/leader_watchlist_2026-08-26.xlsx
+++ b/watchlist_us/leader_watchlist_2026-08-26.xlsx
@@ -772,7 +772,7 @@
         <v>0.1</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.91</v>
+        <v>0.909</v>
       </c>
       <c r="R5" t="n">
         <v>41</v>
@@ -1926,7 +1926,7 @@
         <v>-0.31</v>
       </c>
       <c r="Q23" t="n">
-        <v>0.719</v>
+        <v>0.718</v>
       </c>
       <c r="R23" t="n">
         <v>30</v>
@@ -3091,33 +3091,37 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>SM</t>
+          <t>SNDK</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>SM Energy Company</t>
+          <t>Sandisk</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>에너지</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>마진확장</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
+          <t>시클리컬</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>지금 이익 최고 → 떨어질 수 있음</t>
+        </is>
+      </c>
       <c r="G10" t="n">
-        <v>8.4</v>
+        <v>219.5</v>
       </c>
       <c r="H10" t="n">
-        <v>739</v>
+        <v>57</v>
       </c>
       <c r="I10" t="n">
-        <v>195.9</v>
+        <v>217.2</v>
       </c>
       <c r="J10" t="n">
         <v>3</v>
@@ -3126,28 +3130,28 @@
         <v>83</v>
       </c>
       <c r="L10" t="n">
-        <v>-8.5</v>
+        <v>22.5</v>
       </c>
       <c r="M10" t="n">
-        <v>42.8</v>
+        <v>16.4</v>
       </c>
       <c r="N10" t="n">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="O10" t="n">
-        <v>-132</v>
+        <v>-23</v>
       </c>
       <c r="P10" t="n">
-        <v>4.8</v>
+        <v>63.2</v>
       </c>
       <c r="Q10" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="R10" t="n">
         <v>1.93</v>
       </c>
       <c r="S10" t="n">
-        <v>52</v>
+        <v>115</v>
       </c>
     </row>
     <row r="11">
@@ -3156,37 +3160,33 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>SM</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Sandisk</t>
+          <t>SM Energy Company</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>에너지</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>시클리컬</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>지금 이익 최고 → 떨어질 수 있음</t>
-        </is>
-      </c>
+          <t>마진확장</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
-        <v>219.5</v>
+        <v>8.4</v>
       </c>
       <c r="H11" t="n">
-        <v>57</v>
+        <v>739</v>
       </c>
       <c r="I11" t="n">
-        <v>217.2</v>
+        <v>195.9</v>
       </c>
       <c r="J11" t="n">
         <v>3</v>
@@ -3195,28 +3195,28 @@
         <v>83</v>
       </c>
       <c r="L11" t="n">
-        <v>22.5</v>
+        <v>-8.5</v>
       </c>
       <c r="M11" t="n">
-        <v>16.4</v>
+        <v>42.8</v>
       </c>
       <c r="N11" t="n">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="O11" t="n">
-        <v>-23</v>
+        <v>-132</v>
       </c>
       <c r="P11" t="n">
-        <v>63.2</v>
+        <v>4.8</v>
       </c>
       <c r="Q11" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="R11" t="n">
         <v>1.93</v>
       </c>
       <c r="S11" t="n">
-        <v>115</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12">
@@ -7695,7 +7695,7 @@
         <v>100</v>
       </c>
       <c r="I91" t="n">
-        <v>0.25</v>
+        <v>0.24</v>
       </c>
       <c r="J91" t="n">
         <v>0.66</v>

</xml_diff>